<commit_message>
Updated comorbidity cleaning scripts for both cases and controls, adding new disease classifications
</commit_message>
<xml_diff>
--- a/mgi-analyses/Data-Dictionary.xlsx
+++ b/mgi-analyses/Data-Dictionary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davebrid/Documents/GitHub/ObesityParticulateTreatment/mgi-analyses/cases/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davebrid/Documents/GitHub/ObesityParticulateTreatment/mgi-analyses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227D969A-C393-2A43-AF73-0EBE7AAFE7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDBEBD50-0BA9-F145-9480-675E445FD555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="74">
   <si>
     <t>Type</t>
   </si>
@@ -84,9 +84,6 @@
     <t>DiabetesComplicated, DiabetesUncomplicated</t>
   </si>
   <si>
-    <t>Prior to index case and any, currently any diabetes</t>
-  </si>
-  <si>
     <t>Total Comorbid Score</t>
   </si>
   <si>
@@ -228,48 +225,46 @@
     <t>made in combined_data.Rmd</t>
   </si>
   <si>
-    <t>Type2Diabetes</t>
-  </si>
-  <si>
     <t>DatasetComplete</t>
   </si>
   <si>
     <t>PriorCardiacArrythmia</t>
   </si>
   <si>
-    <t>made in cleaning_comorbidities.Rmd</t>
-  </si>
-  <si>
-    <t>Diabetes: ICD9 CM 250/ICD10-CM-E10 and E11</t>
-  </si>
-  <si>
-    <t>Obesity: ICD9 278/ICD10 CM E66</t>
-  </si>
-  <si>
-    <t>Heart failure: ICD9 428/ICD10 150</t>
-  </si>
-  <si>
-    <t>Chronic kidney disease: ICD9-585 /ICD10-N18</t>
-  </si>
-  <si>
-    <t>Chronic liver disease: ICD9-571/ICD10 K70-K77</t>
-  </si>
-  <si>
-    <t>Dysphagia: ICD9 787.2/ICD10-R13.1 (cause of aspiration pneumonia)</t>
-  </si>
-  <si>
-    <t>Active malignancy:ICD9 40-208/ICD10-C00-C96 (leave out if too complicated)</t>
+    <t>CKD</t>
+  </si>
+  <si>
+    <t>HeartFailure</t>
+  </si>
+  <si>
+    <t>Dysphagia</t>
+  </si>
+  <si>
+    <t>LiverDisease</t>
+  </si>
+  <si>
+    <t>made in both cleaning_comorbidities.Rmd, set to prior to index case or any</t>
+  </si>
+  <si>
+    <t>MetastaticCancer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -303,6 +298,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -324,13 +326,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1002"/>
+  <dimension ref="A1:E1006"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
@@ -614,7 +618,9 @@
       <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="3"/>
+      <c r="E4" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -640,6 +646,9 @@
       <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E6" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
@@ -652,344 +661,389 @@
         <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D14" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>37</v>
+        <v>26</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="B16" s="1" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
-        <v>47</v>
+        <v>35</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="B20" s="1" t="s">
-        <v>49</v>
+        <v>38</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="3"/>
+        <v>42</v>
+      </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="B22" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="B23" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="B24" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>27</v>
+        <v>48</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
+      <c r="B31" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="C31" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E27" s="4" t="s">
+      <c r="C32" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="4" t="s">
+      <c r="D32" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E28" s="4" t="s">
+      <c r="C33" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="4" t="s">
+      <c r="D33" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E29" s="4" t="s">
+      <c r="C34" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="4" t="s">
+      <c r="D34" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E30" s="4" t="s">
+    </row>
+    <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="5"/>
-    </row>
-    <row r="35" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="D35" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="5"/>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="5"/>
+    </row>
+    <row r="38" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="5"/>
+    </row>
+    <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="5"/>
+    </row>
+    <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="5"/>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="5"/>
+    </row>
+    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="5"/>
+    </row>
+    <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="5"/>
+    </row>
+    <row r="44" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1944,6 +1998,10 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1002" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1003" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1004" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1005" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1006" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
Added fields for prior versions of several diseases
</commit_message>
<xml_diff>
--- a/mgi-analyses/Data-Dictionary.xlsx
+++ b/mgi-analyses/Data-Dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davebrid/Documents/GitHub/ObesityParticulateTreatment/mgi-analyses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDBEBD50-0BA9-F145-9480-675E445FD555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20193420-56C8-CA49-B6F0-4C0EFD5EC504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="79">
   <si>
     <t>Type</t>
   </si>
@@ -247,6 +247,21 @@
   </si>
   <si>
     <t>MetastaticCancer</t>
+  </si>
+  <si>
+    <t>PriorLiverDisease</t>
+  </si>
+  <si>
+    <t>PriorMetastaticCancer</t>
+  </si>
+  <si>
+    <t>PriorDysphagia</t>
+  </si>
+  <si>
+    <t>PriorCKD</t>
+  </si>
+  <si>
+    <t>COPD</t>
   </si>
 </sst>
 </file>
@@ -550,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1006"/>
+  <dimension ref="A1:E1007"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
@@ -714,7 +729,7 @@
         <v>53</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>72</v>
@@ -728,7 +743,7 @@
         <v>53</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>72</v>
@@ -742,131 +757,137 @@
         <v>53</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
+    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>39</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>39</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>47</v>
@@ -874,61 +895,61 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="3"/>
-    </row>
-    <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>54</v>
-      </c>
+      <c r="E26" s="3"/>
     </row>
     <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>56</v>
-      </c>
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B29" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>26</v>
@@ -936,38 +957,32 @@
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
+      <c r="B31" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B32" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="4" t="s">
-        <v>62</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>61</v>
+      <c r="D32" s="6" t="s">
+        <v>14</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>65</v>
@@ -975,13 +990,13 @@
     </row>
     <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>61</v>
+      <c r="D33" s="6" t="s">
+        <v>78</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>65</v>
@@ -989,13 +1004,13 @@
     </row>
     <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="4" t="s">
-        <v>61</v>
+      <c r="D34" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>65</v>
@@ -1003,32 +1018,88 @@
     </row>
     <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D35" s="4" t="s">
-        <v>61</v>
+      <c r="D35" s="6" t="s">
+        <v>10</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="5"/>
+      <c r="B36" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="5"/>
+      <c r="B37" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="5"/>
+      <c r="B38" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="5"/>
+      <c r="B39" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="5"/>
+      <c r="B40" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="5"/>
@@ -1039,7 +1110,9 @@
     <row r="43" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="5"/>
     </row>
-    <row r="44" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="5"/>
+    </row>
     <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="46" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="47" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2002,6 +2075,7 @@
     <row r="1004" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1005" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1006" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1007" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>